<commit_message>
implemented the class record and class attendance export excel templates
</commit_message>
<xml_diff>
--- a/Centriku/template/NwSSU-Class-Record.xlsx
+++ b/Centriku/template/NwSSU-Class-Record.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VibeCoding\Centriku\Code\Centriku\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2CFA2D-1D2E-45C7-874B-6E4761B2D0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D12F1D-576E-4F6E-B708-79AE1448E500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="75" yWindow="30" windowWidth="19590" windowHeight="13635" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GENERAL INSTRUCTIONS" sheetId="10" r:id="rId1"/>
@@ -7501,7 +7501,7 @@
         <v/>
       </c>
       <c r="P12" s="97" t="str">
-        <f t="shared" ref="P12:P63" si="0">IFERROR(IF(O12="","",ROUND(O12*$P$11,2)),"")</f>
+        <f>IFERROR(IF(O12="","",ROUND(O12*$P$11,2)),"")</f>
         <v/>
       </c>
       <c r="Q12" s="69"/>
@@ -7555,7 +7555,7 @@
       <c r="L13" s="76"/>
       <c r="M13" s="76"/>
       <c r="N13" s="95" t="str">
-        <f t="shared" ref="N13:N111" si="1">IF(COUNT($D13:$M13)=0,"",SUM($D13:$M13))</f>
+        <f t="shared" ref="N13:N111" si="0">IF(COUNT($D13:$M13)=0,"",SUM($D13:$M13))</f>
         <v/>
       </c>
       <c r="O13" s="96" t="str">
@@ -7563,7 +7563,7 @@
         <v/>
       </c>
       <c r="P13" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="P13:P63" si="1">IFERROR(IF(O13="","",ROUND(O13*$P$11,2)),"")</f>
         <v/>
       </c>
       <c r="Q13" s="69"/>
@@ -7617,7 +7617,7 @@
       <c r="L14" s="76"/>
       <c r="M14" s="76"/>
       <c r="N14" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O14" s="96" t="str">
@@ -7625,7 +7625,7 @@
         <v/>
       </c>
       <c r="P14" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q14" s="69"/>
@@ -7679,7 +7679,7 @@
       <c r="L15" s="76"/>
       <c r="M15" s="76"/>
       <c r="N15" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O15" s="96" t="str">
@@ -7687,7 +7687,7 @@
         <v/>
       </c>
       <c r="P15" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q15" s="69"/>
@@ -7741,7 +7741,7 @@
       <c r="L16" s="76"/>
       <c r="M16" s="76"/>
       <c r="N16" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O16" s="96" t="str">
@@ -7749,7 +7749,7 @@
         <v/>
       </c>
       <c r="P16" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q16" s="69"/>
@@ -7803,7 +7803,7 @@
       <c r="L17" s="76"/>
       <c r="M17" s="76"/>
       <c r="N17" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O17" s="96" t="str">
@@ -7811,7 +7811,7 @@
         <v/>
       </c>
       <c r="P17" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q17" s="69"/>
@@ -7865,7 +7865,7 @@
       <c r="L18" s="76"/>
       <c r="M18" s="76"/>
       <c r="N18" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O18" s="96" t="str">
@@ -7873,7 +7873,7 @@
         <v/>
       </c>
       <c r="P18" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q18" s="69"/>
@@ -7927,7 +7927,7 @@
       <c r="L19" s="76"/>
       <c r="M19" s="76"/>
       <c r="N19" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O19" s="96" t="str">
@@ -7935,7 +7935,7 @@
         <v/>
       </c>
       <c r="P19" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q19" s="69"/>
@@ -7989,7 +7989,7 @@
       <c r="L20" s="76"/>
       <c r="M20" s="76"/>
       <c r="N20" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O20" s="96" t="str">
@@ -7997,7 +7997,7 @@
         <v/>
       </c>
       <c r="P20" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q20" s="69"/>
@@ -8051,7 +8051,7 @@
       <c r="L21" s="76"/>
       <c r="M21" s="76"/>
       <c r="N21" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O21" s="96" t="str">
@@ -8059,7 +8059,7 @@
         <v/>
       </c>
       <c r="P21" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q21" s="69"/>
@@ -8113,7 +8113,7 @@
       <c r="L22" s="76"/>
       <c r="M22" s="76"/>
       <c r="N22" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O22" s="96" t="str">
@@ -8121,7 +8121,7 @@
         <v/>
       </c>
       <c r="P22" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q22" s="69"/>
@@ -8175,7 +8175,7 @@
       <c r="L23" s="76"/>
       <c r="M23" s="76"/>
       <c r="N23" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O23" s="96" t="str">
@@ -8183,7 +8183,7 @@
         <v/>
       </c>
       <c r="P23" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q23" s="69"/>
@@ -8237,7 +8237,7 @@
       <c r="L24" s="76"/>
       <c r="M24" s="76"/>
       <c r="N24" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O24" s="96" t="str">
@@ -8245,7 +8245,7 @@
         <v/>
       </c>
       <c r="P24" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q24" s="69"/>
@@ -8299,7 +8299,7 @@
       <c r="L25" s="76"/>
       <c r="M25" s="76"/>
       <c r="N25" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O25" s="96" t="str">
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="P25" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q25" s="69"/>
@@ -8361,7 +8361,7 @@
       <c r="L26" s="76"/>
       <c r="M26" s="76"/>
       <c r="N26" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O26" s="96" t="str">
@@ -8369,7 +8369,7 @@
         <v/>
       </c>
       <c r="P26" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q26" s="69"/>
@@ -8423,7 +8423,7 @@
       <c r="L27" s="76"/>
       <c r="M27" s="76"/>
       <c r="N27" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O27" s="96" t="str">
@@ -8431,7 +8431,7 @@
         <v/>
       </c>
       <c r="P27" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q27" s="69"/>
@@ -8485,7 +8485,7 @@
       <c r="L28" s="76"/>
       <c r="M28" s="76"/>
       <c r="N28" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O28" s="96" t="str">
@@ -8493,7 +8493,7 @@
         <v/>
       </c>
       <c r="P28" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q28" s="69"/>
@@ -8547,7 +8547,7 @@
       <c r="L29" s="76"/>
       <c r="M29" s="76"/>
       <c r="N29" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O29" s="96" t="str">
@@ -8555,7 +8555,7 @@
         <v/>
       </c>
       <c r="P29" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q29" s="69"/>
@@ -8609,7 +8609,7 @@
       <c r="L30" s="76"/>
       <c r="M30" s="76"/>
       <c r="N30" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O30" s="96" t="str">
@@ -8617,7 +8617,7 @@
         <v/>
       </c>
       <c r="P30" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q30" s="69"/>
@@ -8671,7 +8671,7 @@
       <c r="L31" s="76"/>
       <c r="M31" s="76"/>
       <c r="N31" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O31" s="96" t="str">
@@ -8679,7 +8679,7 @@
         <v/>
       </c>
       <c r="P31" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q31" s="69"/>
@@ -8733,7 +8733,7 @@
       <c r="L32" s="76"/>
       <c r="M32" s="76"/>
       <c r="N32" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O32" s="96" t="str">
@@ -8741,7 +8741,7 @@
         <v/>
       </c>
       <c r="P32" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q32" s="69"/>
@@ -8795,7 +8795,7 @@
       <c r="L33" s="76"/>
       <c r="M33" s="76"/>
       <c r="N33" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O33" s="96" t="str">
@@ -8803,7 +8803,7 @@
         <v/>
       </c>
       <c r="P33" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q33" s="69"/>
@@ -8857,7 +8857,7 @@
       <c r="L34" s="76"/>
       <c r="M34" s="76"/>
       <c r="N34" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O34" s="96" t="str">
@@ -8865,7 +8865,7 @@
         <v/>
       </c>
       <c r="P34" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q34" s="69"/>
@@ -8919,7 +8919,7 @@
       <c r="L35" s="76"/>
       <c r="M35" s="76"/>
       <c r="N35" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O35" s="96" t="str">
@@ -8927,7 +8927,7 @@
         <v/>
       </c>
       <c r="P35" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q35" s="69"/>
@@ -8981,7 +8981,7 @@
       <c r="L36" s="76"/>
       <c r="M36" s="76"/>
       <c r="N36" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O36" s="96" t="str">
@@ -8989,7 +8989,7 @@
         <v/>
       </c>
       <c r="P36" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q36" s="69"/>
@@ -9043,7 +9043,7 @@
       <c r="L37" s="76"/>
       <c r="M37" s="76"/>
       <c r="N37" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O37" s="96" t="str">
@@ -9051,7 +9051,7 @@
         <v/>
       </c>
       <c r="P37" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q37" s="69"/>
@@ -9105,7 +9105,7 @@
       <c r="L38" s="76"/>
       <c r="M38" s="76"/>
       <c r="N38" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O38" s="96" t="str">
@@ -9113,7 +9113,7 @@
         <v/>
       </c>
       <c r="P38" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q38" s="69"/>
@@ -9167,7 +9167,7 @@
       <c r="L39" s="76"/>
       <c r="M39" s="76"/>
       <c r="N39" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O39" s="96" t="str">
@@ -9175,7 +9175,7 @@
         <v/>
       </c>
       <c r="P39" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q39" s="69"/>
@@ -9229,7 +9229,7 @@
       <c r="L40" s="76"/>
       <c r="M40" s="76"/>
       <c r="N40" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O40" s="96" t="str">
@@ -9237,7 +9237,7 @@
         <v/>
       </c>
       <c r="P40" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q40" s="69"/>
@@ -9291,7 +9291,7 @@
       <c r="L41" s="76"/>
       <c r="M41" s="76"/>
       <c r="N41" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O41" s="96" t="str">
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="P41" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q41" s="69"/>
@@ -9353,7 +9353,7 @@
       <c r="L42" s="76"/>
       <c r="M42" s="76"/>
       <c r="N42" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O42" s="96" t="str">
@@ -9361,7 +9361,7 @@
         <v/>
       </c>
       <c r="P42" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q42" s="69"/>
@@ -9415,7 +9415,7 @@
       <c r="L43" s="76"/>
       <c r="M43" s="76"/>
       <c r="N43" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O43" s="96" t="str">
@@ -9423,7 +9423,7 @@
         <v/>
       </c>
       <c r="P43" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q43" s="69"/>
@@ -9477,7 +9477,7 @@
       <c r="L44" s="76"/>
       <c r="M44" s="76"/>
       <c r="N44" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O44" s="96" t="str">
@@ -9485,7 +9485,7 @@
         <v/>
       </c>
       <c r="P44" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q44" s="69"/>
@@ -9539,7 +9539,7 @@
       <c r="L45" s="76"/>
       <c r="M45" s="76"/>
       <c r="N45" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O45" s="96" t="str">
@@ -9547,7 +9547,7 @@
         <v/>
       </c>
       <c r="P45" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q45" s="69"/>
@@ -9601,7 +9601,7 @@
       <c r="L46" s="76"/>
       <c r="M46" s="76"/>
       <c r="N46" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O46" s="96" t="str">
@@ -9609,7 +9609,7 @@
         <v/>
       </c>
       <c r="P46" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q46" s="69"/>
@@ -9663,7 +9663,7 @@
       <c r="L47" s="76"/>
       <c r="M47" s="76"/>
       <c r="N47" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O47" s="96" t="str">
@@ -9671,7 +9671,7 @@
         <v/>
       </c>
       <c r="P47" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q47" s="69"/>
@@ -9725,7 +9725,7 @@
       <c r="L48" s="76"/>
       <c r="M48" s="76"/>
       <c r="N48" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O48" s="96" t="str">
@@ -9733,7 +9733,7 @@
         <v/>
       </c>
       <c r="P48" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q48" s="69"/>
@@ -9787,7 +9787,7 @@
       <c r="L49" s="76"/>
       <c r="M49" s="76"/>
       <c r="N49" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O49" s="96" t="str">
@@ -9795,7 +9795,7 @@
         <v/>
       </c>
       <c r="P49" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q49" s="69"/>
@@ -9849,7 +9849,7 @@
       <c r="L50" s="76"/>
       <c r="M50" s="76"/>
       <c r="N50" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O50" s="96" t="str">
@@ -9857,7 +9857,7 @@
         <v/>
       </c>
       <c r="P50" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q50" s="69"/>
@@ -9911,7 +9911,7 @@
       <c r="L51" s="76"/>
       <c r="M51" s="76"/>
       <c r="N51" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O51" s="96" t="str">
@@ -9919,7 +9919,7 @@
         <v/>
       </c>
       <c r="P51" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q51" s="69"/>
@@ -9973,7 +9973,7 @@
       <c r="L52" s="76"/>
       <c r="M52" s="76"/>
       <c r="N52" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O52" s="96" t="str">
@@ -9981,7 +9981,7 @@
         <v/>
       </c>
       <c r="P52" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q52" s="69"/>
@@ -10035,7 +10035,7 @@
       <c r="L53" s="76"/>
       <c r="M53" s="76"/>
       <c r="N53" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O53" s="96" t="str">
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="P53" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q53" s="69"/>
@@ -10097,7 +10097,7 @@
       <c r="L54" s="76"/>
       <c r="M54" s="76"/>
       <c r="N54" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O54" s="96" t="str">
@@ -10105,7 +10105,7 @@
         <v/>
       </c>
       <c r="P54" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q54" s="69"/>
@@ -10159,7 +10159,7 @@
       <c r="L55" s="76"/>
       <c r="M55" s="76"/>
       <c r="N55" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O55" s="96" t="str">
@@ -10167,7 +10167,7 @@
         <v/>
       </c>
       <c r="P55" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q55" s="69"/>
@@ -10221,7 +10221,7 @@
       <c r="L56" s="76"/>
       <c r="M56" s="76"/>
       <c r="N56" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O56" s="96" t="str">
@@ -10229,7 +10229,7 @@
         <v/>
       </c>
       <c r="P56" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q56" s="69"/>
@@ -10283,7 +10283,7 @@
       <c r="L57" s="76"/>
       <c r="M57" s="76"/>
       <c r="N57" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O57" s="96" t="str">
@@ -10291,7 +10291,7 @@
         <v/>
       </c>
       <c r="P57" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q57" s="69"/>
@@ -10345,7 +10345,7 @@
       <c r="L58" s="76"/>
       <c r="M58" s="76"/>
       <c r="N58" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O58" s="96" t="str">
@@ -10353,7 +10353,7 @@
         <v/>
       </c>
       <c r="P58" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q58" s="69"/>
@@ -10407,7 +10407,7 @@
       <c r="L59" s="76"/>
       <c r="M59" s="76"/>
       <c r="N59" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O59" s="96" t="str">
@@ -10415,7 +10415,7 @@
         <v/>
       </c>
       <c r="P59" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q59" s="69"/>
@@ -10469,7 +10469,7 @@
       <c r="L60" s="76"/>
       <c r="M60" s="76"/>
       <c r="N60" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O60" s="96" t="str">
@@ -10477,7 +10477,7 @@
         <v/>
       </c>
       <c r="P60" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q60" s="69"/>
@@ -10531,7 +10531,7 @@
       <c r="L61" s="76"/>
       <c r="M61" s="76"/>
       <c r="N61" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O61" s="96" t="str">
@@ -10539,7 +10539,7 @@
         <v/>
       </c>
       <c r="P61" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q61" s="69"/>
@@ -10593,7 +10593,7 @@
       <c r="L62" s="76"/>
       <c r="M62" s="76"/>
       <c r="N62" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O62" s="96" t="str">
@@ -10601,7 +10601,7 @@
         <v/>
       </c>
       <c r="P62" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q62" s="69"/>
@@ -10655,7 +10655,7 @@
       <c r="L63" s="76"/>
       <c r="M63" s="76"/>
       <c r="N63" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O63" s="96" t="str">
@@ -10663,7 +10663,7 @@
         <v/>
       </c>
       <c r="P63" s="97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q63" s="69"/>
@@ -10717,7 +10717,7 @@
       <c r="L64" s="76"/>
       <c r="M64" s="76"/>
       <c r="N64" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O64" s="96" t="str">
@@ -10779,7 +10779,7 @@
       <c r="L65" s="76"/>
       <c r="M65" s="76"/>
       <c r="N65" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O65" s="96" t="str">
@@ -10841,7 +10841,7 @@
       <c r="L66" s="76"/>
       <c r="M66" s="76"/>
       <c r="N66" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O66" s="96" t="str">
@@ -10903,7 +10903,7 @@
       <c r="L67" s="76"/>
       <c r="M67" s="76"/>
       <c r="N67" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O67" s="96" t="str">
@@ -10965,7 +10965,7 @@
       <c r="L68" s="76"/>
       <c r="M68" s="76"/>
       <c r="N68" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O68" s="96" t="str">
@@ -11027,7 +11027,7 @@
       <c r="L69" s="76"/>
       <c r="M69" s="76"/>
       <c r="N69" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O69" s="96" t="str">
@@ -11089,7 +11089,7 @@
       <c r="L70" s="76"/>
       <c r="M70" s="76"/>
       <c r="N70" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O70" s="96" t="str">
@@ -11151,7 +11151,7 @@
       <c r="L71" s="76"/>
       <c r="M71" s="76"/>
       <c r="N71" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O71" s="96" t="str">
@@ -11213,7 +11213,7 @@
       <c r="L72" s="76"/>
       <c r="M72" s="76"/>
       <c r="N72" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O72" s="96" t="str">
@@ -11275,7 +11275,7 @@
       <c r="L73" s="76"/>
       <c r="M73" s="76"/>
       <c r="N73" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O73" s="96" t="str">
@@ -11337,7 +11337,7 @@
       <c r="L74" s="76"/>
       <c r="M74" s="76"/>
       <c r="N74" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O74" s="96" t="str">
@@ -11399,7 +11399,7 @@
       <c r="L75" s="76"/>
       <c r="M75" s="76"/>
       <c r="N75" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O75" s="96" t="str">
@@ -11461,7 +11461,7 @@
       <c r="L76" s="76"/>
       <c r="M76" s="76"/>
       <c r="N76" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O76" s="96" t="str">
@@ -11523,7 +11523,7 @@
       <c r="L77" s="76"/>
       <c r="M77" s="76"/>
       <c r="N77" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O77" s="96" t="str">
@@ -11585,7 +11585,7 @@
       <c r="L78" s="76"/>
       <c r="M78" s="76"/>
       <c r="N78" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O78" s="96" t="str">
@@ -11647,7 +11647,7 @@
       <c r="L79" s="76"/>
       <c r="M79" s="76"/>
       <c r="N79" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O79" s="96" t="str">
@@ -11709,7 +11709,7 @@
       <c r="L80" s="76"/>
       <c r="M80" s="76"/>
       <c r="N80" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O80" s="96" t="str">
@@ -11771,7 +11771,7 @@
       <c r="L81" s="76"/>
       <c r="M81" s="76"/>
       <c r="N81" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O81" s="96" t="str">
@@ -11833,7 +11833,7 @@
       <c r="L82" s="76"/>
       <c r="M82" s="76"/>
       <c r="N82" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O82" s="96" t="str">
@@ -11895,7 +11895,7 @@
       <c r="L83" s="76"/>
       <c r="M83" s="76"/>
       <c r="N83" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O83" s="96" t="str">
@@ -11957,7 +11957,7 @@
       <c r="L84" s="76"/>
       <c r="M84" s="76"/>
       <c r="N84" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O84" s="96" t="str">
@@ -12019,7 +12019,7 @@
       <c r="L85" s="76"/>
       <c r="M85" s="76"/>
       <c r="N85" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O85" s="96" t="str">
@@ -12081,7 +12081,7 @@
       <c r="L86" s="76"/>
       <c r="M86" s="76"/>
       <c r="N86" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O86" s="96" t="str">
@@ -12143,7 +12143,7 @@
       <c r="L87" s="76"/>
       <c r="M87" s="76"/>
       <c r="N87" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O87" s="96" t="str">
@@ -12205,7 +12205,7 @@
       <c r="L88" s="76"/>
       <c r="M88" s="76"/>
       <c r="N88" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O88" s="96" t="str">
@@ -12267,7 +12267,7 @@
       <c r="L89" s="76"/>
       <c r="M89" s="76"/>
       <c r="N89" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O89" s="96" t="str">
@@ -12329,7 +12329,7 @@
       <c r="L90" s="76"/>
       <c r="M90" s="76"/>
       <c r="N90" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O90" s="96" t="str">
@@ -12391,7 +12391,7 @@
       <c r="L91" s="76"/>
       <c r="M91" s="76"/>
       <c r="N91" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O91" s="96" t="str">
@@ -12453,7 +12453,7 @@
       <c r="L92" s="76"/>
       <c r="M92" s="76"/>
       <c r="N92" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O92" s="96" t="str">
@@ -12515,7 +12515,7 @@
       <c r="L93" s="76"/>
       <c r="M93" s="76"/>
       <c r="N93" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O93" s="96" t="str">
@@ -12577,7 +12577,7 @@
       <c r="L94" s="76"/>
       <c r="M94" s="76"/>
       <c r="N94" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O94" s="96" t="str">
@@ -12639,7 +12639,7 @@
       <c r="L95" s="76"/>
       <c r="M95" s="76"/>
       <c r="N95" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O95" s="96" t="str">
@@ -12701,7 +12701,7 @@
       <c r="L96" s="76"/>
       <c r="M96" s="76"/>
       <c r="N96" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O96" s="96" t="str">
@@ -12763,7 +12763,7 @@
       <c r="L97" s="76"/>
       <c r="M97" s="76"/>
       <c r="N97" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O97" s="96" t="str">
@@ -12825,7 +12825,7 @@
       <c r="L98" s="76"/>
       <c r="M98" s="76"/>
       <c r="N98" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O98" s="96" t="str">
@@ -12887,7 +12887,7 @@
       <c r="L99" s="76"/>
       <c r="M99" s="76"/>
       <c r="N99" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O99" s="96" t="str">
@@ -12949,7 +12949,7 @@
       <c r="L100" s="76"/>
       <c r="M100" s="76"/>
       <c r="N100" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O100" s="96" t="str">
@@ -13011,7 +13011,7 @@
       <c r="L101" s="76"/>
       <c r="M101" s="76"/>
       <c r="N101" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O101" s="96" t="str">
@@ -13073,7 +13073,7 @@
       <c r="L102" s="76"/>
       <c r="M102" s="76"/>
       <c r="N102" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O102" s="96" t="str">
@@ -13135,7 +13135,7 @@
       <c r="L103" s="76"/>
       <c r="M103" s="76"/>
       <c r="N103" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O103" s="96" t="str">
@@ -13197,7 +13197,7 @@
       <c r="L104" s="76"/>
       <c r="M104" s="76"/>
       <c r="N104" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O104" s="96" t="str">
@@ -13259,7 +13259,7 @@
       <c r="L105" s="76"/>
       <c r="M105" s="76"/>
       <c r="N105" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O105" s="96" t="str">
@@ -13321,7 +13321,7 @@
       <c r="L106" s="76"/>
       <c r="M106" s="76"/>
       <c r="N106" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O106" s="96" t="str">
@@ -13383,7 +13383,7 @@
       <c r="L107" s="76"/>
       <c r="M107" s="76"/>
       <c r="N107" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O107" s="96" t="str">
@@ -13445,7 +13445,7 @@
       <c r="L108" s="76"/>
       <c r="M108" s="76"/>
       <c r="N108" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O108" s="96" t="str">
@@ -13507,7 +13507,7 @@
       <c r="L109" s="76"/>
       <c r="M109" s="76"/>
       <c r="N109" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O109" s="96" t="str">
@@ -13569,7 +13569,7 @@
       <c r="L110" s="76"/>
       <c r="M110" s="76"/>
       <c r="N110" s="95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O110" s="96" t="str">
@@ -13631,7 +13631,7 @@
       <c r="L111" s="80"/>
       <c r="M111" s="80"/>
       <c r="N111" s="100" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="O111" s="101" t="str">
@@ -13675,7 +13675,7 @@
       <c r="AC111" s="55"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="72Fg3wg5QPqDpvXIY8CwzN6V6EDJx6KunMI2PoJbOsh/8WUc3XJmQu3fxZ7Bp+m19iziIVdVzNFSsN3YRXAStg==" saltValue="oqM55QGGEBdU0RNPBHjq6Q==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="26">
     <mergeCell ref="I2:W2"/>
     <mergeCell ref="I3:W3"/>
@@ -20674,10 +20674,7 @@
         <f>'FINAL TERM'!AB12</f>
         <v/>
       </c>
-      <c r="G12" s="31" t="str">
-        <f>IF(OR(E12="",F12=""),"",IF(ISERROR(ROUND(AVERAGE(E12,F12),0)),"",ROUND(AVERAGE(E12,F12),0)))</f>
-        <v/>
-      </c>
+      <c r="G12" s="31"/>
       <c r="H12" s="31" t="str">
         <f>IF(G12="","",IF(G12=100,"1.00",IF(G12=99,"1.00",IF(G12=98,"1.00",IF(G12=97,"1.00",IF(G12=96,"1.00",IF(G12=96,"1.00",IF(G12=95,"1.00",IF(G12=94,"1.10",IF(G12=93,"1.20",IF(G12=92,"1.30",IF(G12=91,"1.40",IF(G12=90,"1.50",IF(G12=89,"1.60",IF(G12=88,"1.70",IF(G12=87,"1.80",IF(G12=86,"1.90",IF(G12=85,"2.00",IF(G12=84,"2.10",IF(G12=83,"2.20",IF(G12=82,"2.30",IF(G12=81,"2.40",IF(G12=80,"2.50",IF(G12=79,"2.60",IF(G12=78,"2.70",IF(G12=77,"2.80",IF(G12=76,"2.90",IF(G12=75,"3.00",IF(G12&lt;75,"5.00")))))))))))))))))))))))))))))</f>
         <v/>
@@ -25055,7 +25052,7 @@
       <c r="T111" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="izDf/WVhJGYwJtOE/xcLMFkFrzKRFPoFhqld27EV1VbnF6O4JLg295n8ExJhlOX3DcyxTMhzeasvIShAsCtuiw==" saltValue="OlS0Pq0wB/8I3xW3Q5lLsg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="23">
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B3:I3"/>

</xml_diff>